<commit_message>
Atualiza dashboard e painel de motos
</commit_message>
<xml_diff>
--- a/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
+++ b/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
@@ -42,7 +42,7 @@
     <t>MANUTENÇÃO PREVENTIVA</t>
   </si>
   <si>
-    <t>1000 km restantes</t>
+    <t>965 km restantes</t>
   </si>
   <si>
     <t>TROCA DE OLEO</t>
@@ -51,22 +51,22 @@
     <t>FNP-0372</t>
   </si>
   <si>
-    <t>999 km restantes</t>
+    <t>974 km restantes</t>
   </si>
   <si>
     <t>FNP-4083</t>
   </si>
   <si>
-    <t>9999 km restantes</t>
+    <t>9627 km restantes</t>
   </si>
   <si>
     <t>FNP-4094</t>
   </si>
   <si>
-    <t>7655 km restantes</t>
-  </si>
-  <si>
-    <t>37655 km restantes</t>
+    <t>7619 km restantes</t>
+  </si>
+  <si>
+    <t>37619 km restantes</t>
   </si>
   <si>
     <t>RODAGEM DE PNEUS</t>
@@ -75,19 +75,19 @@
     <t>FNP-4100</t>
   </si>
   <si>
-    <t>4745 km expirado</t>
-  </si>
-  <si>
-    <t>25255 km restantes</t>
+    <t>5018 km expirado</t>
+  </si>
+  <si>
+    <t>24982 km restantes</t>
   </si>
   <si>
     <t>FNP-4103</t>
   </si>
   <si>
-    <t>4107 km expirado</t>
-  </si>
-  <si>
-    <t>25893 km restantes</t>
+    <t>19496 km expirado</t>
+  </si>
+  <si>
+    <t>10504 km restantes</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Atualiza Central de Monitoramento Frotas Leves
</commit_message>
<xml_diff>
--- a/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
+++ b/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
@@ -51,22 +51,22 @@
     <t>FNP-0372</t>
   </si>
   <si>
-    <t>974 km restantes</t>
+    <t>901 km restantes</t>
   </si>
   <si>
     <t>FNP-4083</t>
   </si>
   <si>
-    <t>9627 km restantes</t>
+    <t>9404 km restantes</t>
   </si>
   <si>
     <t>FNP-4094</t>
   </si>
   <si>
-    <t>7619 km restantes</t>
-  </si>
-  <si>
-    <t>37619 km restantes</t>
+    <t>7478 km restantes</t>
+  </si>
+  <si>
+    <t>37478 km restantes</t>
   </si>
   <si>
     <t>RODAGEM DE PNEUS</t>
@@ -75,19 +75,19 @@
     <t>FNP-4100</t>
   </si>
   <si>
-    <t>5018 km expirado</t>
-  </si>
-  <si>
-    <t>24982 km restantes</t>
+    <t>5237 km expirado</t>
+  </si>
+  <si>
+    <t>24763 km restantes</t>
   </si>
   <si>
     <t>FNP-4103</t>
   </si>
   <si>
-    <t>19496 km expirado</t>
-  </si>
-  <si>
-    <t>10504 km restantes</t>
+    <t>19552 km expirado</t>
+  </si>
+  <si>
+    <t>10448 km restantes</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Atualiza bases e protege acesso ao dashboard
</commit_message>
<xml_diff>
--- a/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
+++ b/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
@@ -51,22 +51,22 @@
     <t>FNP-0372</t>
   </si>
   <si>
-    <t>901 km restantes</t>
+    <t>892 km restantes</t>
   </si>
   <si>
     <t>FNP-4083</t>
   </si>
   <si>
-    <t>9404 km restantes</t>
+    <t>9279 km restantes</t>
   </si>
   <si>
     <t>FNP-4094</t>
   </si>
   <si>
-    <t>7478 km restantes</t>
-  </si>
-  <si>
-    <t>37478 km restantes</t>
+    <t>7296 km restantes</t>
+  </si>
+  <si>
+    <t>37296 km restantes</t>
   </si>
   <si>
     <t>RODAGEM DE PNEUS</t>
@@ -75,19 +75,19 @@
     <t>FNP-4100</t>
   </si>
   <si>
-    <t>5237 km expirado</t>
-  </si>
-  <si>
-    <t>24763 km restantes</t>
+    <t>5369 km expirado</t>
+  </si>
+  <si>
+    <t>24631 km restantes</t>
   </si>
   <si>
     <t>FNP-4103</t>
   </si>
   <si>
-    <t>19552 km expirado</t>
-  </si>
-  <si>
-    <t>10448 km restantes</t>
+    <t>19687 km expirado</t>
+  </si>
+  <si>
+    <t>10313 km restantes</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Adicionar filtros estilo Excel nas tabelas
</commit_message>
<xml_diff>
--- a/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
+++ b/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
@@ -51,22 +51,22 @@
     <t>FNP-0372</t>
   </si>
   <si>
-    <t>892 km restantes</t>
+    <t>804 km restantes</t>
   </si>
   <si>
     <t>FNP-4083</t>
   </si>
   <si>
-    <t>9279 km restantes</t>
+    <t>7392 km restantes</t>
   </si>
   <si>
     <t>FNP-4094</t>
   </si>
   <si>
-    <t>7296 km restantes</t>
-  </si>
-  <si>
-    <t>37296 km restantes</t>
+    <t>4985 km restantes</t>
+  </si>
+  <si>
+    <t>34985 km restantes</t>
   </si>
   <si>
     <t>RODAGEM DE PNEUS</t>
@@ -75,19 +75,19 @@
     <t>FNP-4100</t>
   </si>
   <si>
-    <t>5369 km expirado</t>
-  </si>
-  <si>
-    <t>24631 km restantes</t>
+    <t>5928 km expirado</t>
+  </si>
+  <si>
+    <t>24072 km restantes</t>
   </si>
   <si>
     <t>FNP-4103</t>
   </si>
   <si>
-    <t>19687 km expirado</t>
-  </si>
-  <si>
-    <t>10313 km restantes</t>
+    <t>19353 km restantes</t>
+  </si>
+  <si>
+    <t>49353 km restantes</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Atualiza dashboard SuperRota e prepara publicacao
</commit_message>
<xml_diff>
--- a/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
+++ b/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
@@ -51,22 +51,22 @@
     <t>FNP-0372</t>
   </si>
   <si>
-    <t>804 km restantes</t>
+    <t>842 km restantes</t>
   </si>
   <si>
     <t>FNP-4083</t>
   </si>
   <si>
-    <t>7392 km restantes</t>
+    <t>9226 km restantes</t>
   </si>
   <si>
     <t>FNP-4094</t>
   </si>
   <si>
-    <t>4985 km restantes</t>
-  </si>
-  <si>
-    <t>34985 km restantes</t>
+    <t>5196 km restantes</t>
+  </si>
+  <si>
+    <t>35196 km restantes</t>
   </si>
   <si>
     <t>RODAGEM DE PNEUS</t>
@@ -75,19 +75,19 @@
     <t>FNP-4100</t>
   </si>
   <si>
-    <t>5928 km expirado</t>
-  </si>
-  <si>
-    <t>24072 km restantes</t>
+    <t>5649 km expirado</t>
+  </si>
+  <si>
+    <t>24351 km restantes</t>
   </si>
   <si>
     <t>FNP-4103</t>
   </si>
   <si>
-    <t>19353 km restantes</t>
-  </si>
-  <si>
-    <t>49353 km restantes</t>
+    <t>19550 km restantes</t>
+  </si>
+  <si>
+    <t>49550 km restantes</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Atualizacao SuperRota 30/08/2026 11:19:02,59
</commit_message>
<xml_diff>
--- a/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
+++ b/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
@@ -42,7 +42,7 @@
     <t>MANUTENÇÃO PREVENTIVA</t>
   </si>
   <si>
-    <t>965 km restantes</t>
+    <t>964 km restantes</t>
   </si>
   <si>
     <t>TROCA DE OLEO</t>
@@ -51,22 +51,22 @@
     <t>FNP-0372</t>
   </si>
   <si>
-    <t>842 km restantes</t>
+    <t>745 km restantes</t>
   </si>
   <si>
     <t>FNP-4083</t>
   </si>
   <si>
-    <t>9226 km restantes</t>
+    <t>7027 km restantes</t>
   </si>
   <si>
     <t>FNP-4094</t>
   </si>
   <si>
-    <t>5196 km restantes</t>
-  </si>
-  <si>
-    <t>35196 km restantes</t>
+    <t>4904 km restantes</t>
+  </si>
+  <si>
+    <t>34904 km restantes</t>
   </si>
   <si>
     <t>RODAGEM DE PNEUS</t>
@@ -75,19 +75,19 @@
     <t>FNP-4100</t>
   </si>
   <si>
-    <t>5649 km expirado</t>
-  </si>
-  <si>
-    <t>24351 km restantes</t>
+    <t>6267 km expirado</t>
+  </si>
+  <si>
+    <t>23733 km restantes</t>
   </si>
   <si>
     <t>FNP-4103</t>
   </si>
   <si>
-    <t>19550 km restantes</t>
-  </si>
-  <si>
-    <t>49550 km restantes</t>
+    <t>2050 km restantes</t>
+  </si>
+  <si>
+    <t>32050 km restantes</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Atualizacao SuperRota 02/09/2026  9:02:21,75
</commit_message>
<xml_diff>
--- a/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
+++ b/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
@@ -42,7 +42,7 @@
     <t>MANUTENÇÃO PREVENTIVA</t>
   </si>
   <si>
-    <t>964 km restantes</t>
+    <t>962 km restantes</t>
   </si>
   <si>
     <t>TROCA DE OLEO</t>
@@ -51,22 +51,22 @@
     <t>FNP-0372</t>
   </si>
   <si>
-    <t>745 km restantes</t>
+    <t>677 km restantes</t>
   </si>
   <si>
     <t>FNP-4083</t>
   </si>
   <si>
-    <t>7027 km restantes</t>
+    <t>6878 km restantes</t>
   </si>
   <si>
     <t>FNP-4094</t>
   </si>
   <si>
-    <t>4904 km restantes</t>
-  </si>
-  <si>
-    <t>34904 km restantes</t>
+    <t>4850 km restantes</t>
+  </si>
+  <si>
+    <t>34850 km restantes</t>
   </si>
   <si>
     <t>RODAGEM DE PNEUS</t>
@@ -75,19 +75,19 @@
     <t>FNP-4100</t>
   </si>
   <si>
-    <t>6267 km expirado</t>
-  </si>
-  <si>
-    <t>23733 km restantes</t>
+    <t>25342 km expirado</t>
+  </si>
+  <si>
+    <t>4658 km restantes</t>
   </si>
   <si>
     <t>FNP-4103</t>
   </si>
   <si>
-    <t>2050 km restantes</t>
-  </si>
-  <si>
-    <t>32050 km restantes</t>
+    <t>1625 km restantes</t>
+  </si>
+  <si>
+    <t>31625 km restantes</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Atualizacao SuperRota 08/09/2026  7:13:21,54
</commit_message>
<xml_diff>
--- a/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
+++ b/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
@@ -51,22 +51,22 @@
     <t>FNP-0372</t>
   </si>
   <si>
-    <t>677 km restantes</t>
+    <t>561 km restantes</t>
   </si>
   <si>
     <t>FNP-4083</t>
   </si>
   <si>
-    <t>6878 km restantes</t>
+    <t>2570 km restantes</t>
   </si>
   <si>
     <t>FNP-4094</t>
   </si>
   <si>
-    <t>4850 km restantes</t>
-  </si>
-  <si>
-    <t>34850 km restantes</t>
+    <t>834 km restantes</t>
+  </si>
+  <si>
+    <t>30834 km restantes</t>
   </si>
   <si>
     <t>RODAGEM DE PNEUS</t>
@@ -75,26 +75,26 @@
     <t>FNP-4100</t>
   </si>
   <si>
-    <t>25342 km expirado</t>
-  </si>
-  <si>
-    <t>4658 km restantes</t>
+    <t>26159 km expirado</t>
+  </si>
+  <si>
+    <t>3841 km restantes</t>
   </si>
   <si>
     <t>FNP-4103</t>
   </si>
   <si>
-    <t>1625 km restantes</t>
-  </si>
-  <si>
-    <t>31625 km restantes</t>
+    <t>17874 km expirado</t>
+  </si>
+  <si>
+    <t>12126 km restantes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="43">
+  <numFmts count="44">
     <numFmt formatCode="#0" numFmtId="0"/>
     <numFmt formatCode="#0" numFmtId="1"/>
     <numFmt formatCode="0.0" numFmtId="2"/>
@@ -102,42 +102,43 @@
     <numFmt formatCode="0.#0" numFmtId="4"/>
     <numFmt formatCode="#0" numFmtId="5"/>
     <numFmt formatCode="DD.MM.YYYY HH:MM:SS" numFmtId="6"/>
-    <numFmt formatCode="DD.MM.YYYY" numFmtId="7"/>
-    <numFmt formatCode="HH:MM:SS" numFmtId="8"/>
-    <numFmt formatCode="[H]&quot; horas &quot;M&quot; minutos&quot;" numFmtId="9"/>
+    <numFmt formatCode="DD.MM.YYYY HH:MM:SS" numFmtId="7"/>
+    <numFmt formatCode="DD.MM.YYYY" numFmtId="8"/>
+    <numFmt formatCode="HH:MM:SS" numFmtId="9"/>
     <numFmt formatCode="[H]&quot; horas &quot;M&quot; minutos&quot;" numFmtId="10"/>
-    <numFmt formatCode="0.#0" numFmtId="11"/>
+    <numFmt formatCode="[H]&quot; horas &quot;M&quot; minutos&quot;" numFmtId="11"/>
     <numFmt formatCode="0.#0" numFmtId="12"/>
-    <numFmt formatCode="#0" numFmtId="13"/>
-    <numFmt formatCode="#0&quot; km&quot;" numFmtId="14"/>
+    <numFmt formatCode="0.#0" numFmtId="13"/>
+    <numFmt formatCode="#0" numFmtId="14"/>
     <numFmt formatCode="#0&quot; km&quot;" numFmtId="15"/>
-    <numFmt formatCode="#0&quot; km/h&quot;" numFmtId="16"/>
+    <numFmt formatCode="#0&quot; km&quot;" numFmtId="16"/>
     <numFmt formatCode="#0&quot; km/h&quot;" numFmtId="17"/>
-    <numFmt formatCode="#0&quot; l&quot;" numFmtId="18"/>
+    <numFmt formatCode="#0&quot; km/h&quot;" numFmtId="18"/>
     <numFmt formatCode="#0&quot; l&quot;" numFmtId="19"/>
-    <numFmt formatCode="#0&quot; l/100 km&quot;" numFmtId="20"/>
-    <numFmt formatCode="#0 &quot;l/h&quot;" numFmtId="21"/>
-    <numFmt formatCode="0.0&quot;%&quot;" numFmtId="22"/>
+    <numFmt formatCode="#0&quot; l&quot;" numFmtId="20"/>
+    <numFmt formatCode="#0&quot; l/100 km&quot;" numFmtId="21"/>
+    <numFmt formatCode="#0 &quot;l/h&quot;" numFmtId="22"/>
     <numFmt formatCode="0.0&quot;%&quot;" numFmtId="23"/>
-    <numFmt formatCode="0.#0&quot; ha&quot;" numFmtId="24"/>
-    <numFmt formatCode="#0&quot; °C&quot;" numFmtId="25"/>
-    <numFmt formatCode="0.#0&quot; km&quot;" numFmtId="26"/>
+    <numFmt formatCode="0.0&quot;%&quot;" numFmtId="24"/>
+    <numFmt formatCode="0.#0&quot; ha&quot;" numFmtId="25"/>
+    <numFmt formatCode="#0&quot; °C&quot;" numFmtId="26"/>
     <numFmt formatCode="0.#0&quot; km&quot;" numFmtId="27"/>
     <numFmt formatCode="0.#0&quot; km&quot;" numFmtId="28"/>
-    <numFmt formatCode="0.#0&quot; l&quot;" numFmtId="29"/>
+    <numFmt formatCode="0.#0&quot; km&quot;" numFmtId="29"/>
     <numFmt formatCode="0.#0&quot; l&quot;" numFmtId="30"/>
-    <numFmt formatCode="0.#0&quot; l/100 km&quot;" numFmtId="31"/>
-    <numFmt formatCode="0.#0 &quot;l/h&quot;" numFmtId="32"/>
-    <numFmt formatCode="0.#0&quot; B&quot;" numFmtId="33"/>
-    <numFmt formatCode="0.#0&quot; KB&quot;" numFmtId="34"/>
-    <numFmt formatCode="0.#0&quot; MB&quot;" numFmtId="35"/>
-    <numFmt formatCode="0.#0 &quot;t&quot;" numFmtId="36"/>
-    <numFmt formatCode="0.#00 &quot;t&quot;" numFmtId="37"/>
-    <numFmt formatCode="0.#000 &quot;t&quot;" numFmtId="38"/>
-    <numFmt formatCode="0.#0&quot; m&quot;" numFmtId="39"/>
-    <numFmt formatCode="0.#0&quot; km&quot;" numFmtId="40"/>
-    <numFmt formatCode="0.#0&quot; ha&quot;" numFmtId="41"/>
-    <numFmt formatCode="0.#0&quot; mi²&quot;" numFmtId="42"/>
+    <numFmt formatCode="0.#0&quot; l&quot;" numFmtId="31"/>
+    <numFmt formatCode="0.#0&quot; l/100 km&quot;" numFmtId="32"/>
+    <numFmt formatCode="0.#0 &quot;l/h&quot;" numFmtId="33"/>
+    <numFmt formatCode="0.#0&quot; B&quot;" numFmtId="34"/>
+    <numFmt formatCode="0.#0&quot; KB&quot;" numFmtId="35"/>
+    <numFmt formatCode="0.#0&quot; MB&quot;" numFmtId="36"/>
+    <numFmt formatCode="0.#0 &quot;t&quot;" numFmtId="37"/>
+    <numFmt formatCode="0.#00 &quot;t&quot;" numFmtId="38"/>
+    <numFmt formatCode="0.#000 &quot;t&quot;" numFmtId="39"/>
+    <numFmt formatCode="0.#0&quot; m&quot;" numFmtId="40"/>
+    <numFmt formatCode="0.#0&quot; km&quot;" numFmtId="41"/>
+    <numFmt formatCode="0.#0&quot; ha&quot;" numFmtId="42"/>
+    <numFmt formatCode="0.#0&quot; mi²&quot;" numFmtId="43"/>
   </numFmts>
   <fonts count="2">
     <font>

</xml_diff>

<commit_message>
Atualizacao SuperRota 11/09/2026 14:49:17,50
</commit_message>
<xml_diff>
--- a/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
+++ b/dados/FNP-_Manuten#U00e7#U00f5es_-_Grupo_21.08.2026_13-53-59.xlsx
@@ -51,22 +51,22 @@
     <t>FNP-0372</t>
   </si>
   <si>
-    <t>561 km restantes</t>
+    <t>526 km restantes</t>
   </si>
   <si>
     <t>FNP-4083</t>
   </si>
   <si>
-    <t>2570 km restantes</t>
+    <t>2979 km expirado</t>
   </si>
   <si>
     <t>FNP-4094</t>
   </si>
   <si>
-    <t>834 km restantes</t>
-  </si>
-  <si>
-    <t>30834 km restantes</t>
+    <t>558 km restantes</t>
+  </si>
+  <si>
+    <t>30558 km restantes</t>
   </si>
   <si>
     <t>RODAGEM DE PNEUS</t>
@@ -75,19 +75,19 @@
     <t>FNP-4100</t>
   </si>
   <si>
-    <t>26159 km expirado</t>
-  </si>
-  <si>
-    <t>3841 km restantes</t>
+    <t>26804 km expirado</t>
+  </si>
+  <si>
+    <t>3196 km restantes</t>
   </si>
   <si>
     <t>FNP-4103</t>
   </si>
   <si>
-    <t>17874 km expirado</t>
-  </si>
-  <si>
-    <t>12126 km restantes</t>
+    <t>18055 km expirado</t>
+  </si>
+  <si>
+    <t>11945 km restantes</t>
   </si>
 </sst>
 </file>

</xml_diff>